<commit_message>
commit new excel file
</commit_message>
<xml_diff>
--- a/Release_Readiness_Score.xlsx
+++ b/Release_Readiness_Score.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="43">
   <si>
     <t>RELEASE READINESS SCORE REPORT</t>
   </si>
   <si>
-    <t>Generated: 4/6/2026, 11:20:53 am</t>
+    <t>Generated: 5/6/2026, 11:54:05 am</t>
   </si>
   <si>
     <t>OVERALL METRICS</t>
@@ -45,27 +45,21 @@
     <t>Tests Passed</t>
   </si>
   <si>
-    <t>⚠</t>
-  </si>
-  <si>
-    <t>89.29%</t>
+    <t>✓</t>
+  </si>
+  <si>
+    <t>100%</t>
   </si>
   <si>
     <t>Tests Failed</t>
   </si>
   <si>
-    <t>✗</t>
-  </si>
-  <si>
-    <t>10.71%</t>
+    <t>0%</t>
   </si>
   <si>
     <t>Tests with Errors</t>
   </si>
   <si>
-    <t>✓</t>
-  </si>
-  <si>
     <t>Critical</t>
   </si>
   <si>
@@ -75,16 +69,13 @@
     <t>Test Coverage</t>
   </si>
   <si>
-    <t>100%</t>
-  </si>
-  <si>
-    <t>28 active</t>
+    <t>26 active</t>
   </si>
   <si>
     <t>Total Execution Time</t>
   </si>
   <si>
-    <t>137.66s</t>
+    <t>79.43s</t>
   </si>
   <si>
     <t>Performance metric</t>
@@ -96,13 +87,13 @@
     <t>Primary KPI</t>
   </si>
   <si>
-    <t>RELEASE READINESS SCORE: 94.64/100</t>
+    <t>RELEASE READINESS SCORE: 100/100</t>
   </si>
   <si>
     <t>QUALITY GRADE: A - Production Ready</t>
   </si>
   <si>
-    <t>RECOMMENDATION: ✓ READY FOR RELEASE - Minor monitoring recommended</t>
+    <t>RECOMMENDATION: ✓ APPROVED FOR PRODUCTION - All systems go!</t>
   </si>
   <si>
     <t>TEST SUITE BREAKDOWN</t>
@@ -144,26 +135,20 @@
     <t>RISK ASSESSMENT &amp; RECOMMENDATIONS</t>
   </si>
   <si>
-    <t>Test Failures</t>
-  </si>
-  <si>
-    <t>HIGH</t>
-  </si>
-  <si>
-    <t>3 test(s) failed. Investigate and fix before release.</t>
-  </si>
-  <si>
-    <t>MEDIUM</t>
-  </si>
-  <si>
-    <t>Pass rate is 89.29%. Target should be &gt;= 90% for production release.</t>
+    <t>Overall Status</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>No critical risks identified. System appears ready for release.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -191,14 +176,6 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF9C6500"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF9C0006"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FF006100"/>
     </font>
     <font>
@@ -215,7 +192,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -239,16 +216,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
@@ -259,12 +226,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor rgb="FF92D050"/>
       </patternFill>
     </fill>
   </fills>
@@ -280,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -289,27 +251,22 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -698,7 +655,7 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
         <v>8</v>
@@ -712,7 +669,7 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>10</v>
@@ -726,32 +683,32 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>3</v>
-      </c>
-      <c r="C8" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" t="s">
         <v>13</v>
-      </c>
-      <c r="D8" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" t="s">
         <v>15</v>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -765,35 +722,35 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>16</v>
+        <v>11</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>16</v>
+        <v>20</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>10</v>
       </c>
       <c r="D12" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
@@ -802,32 +759,32 @@
         <v>10</v>
       </c>
       <c r="D13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+    </row>
+    <row r="17" ht="25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="16" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-    </row>
-    <row r="17" ht="25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -857,38 +814,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="D2" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="E2" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="F2" s="10" t="s">
         <v>33</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B3">
         <v>7</v>
@@ -902,13 +859,13 @@
       <c r="E3">
         <v>0</v>
       </c>
-      <c r="F3" s="13">
+      <c r="F3" s="11">
         <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B4">
         <v>6</v>
@@ -922,13 +879,13 @@
       <c r="E4">
         <v>0</v>
       </c>
-      <c r="F4" s="13">
+      <c r="F4" s="11">
         <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B5">
         <v>6</v>
@@ -942,48 +899,48 @@
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5" s="13">
+      <c r="F5" s="11">
         <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C6">
         <v>2</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6" s="14">
-        <v>50</v>
+      <c r="F6" s="11">
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B7">
         <v>5</v>
       </c>
       <c r="C7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
-      <c r="F7" s="15">
-        <v>80</v>
+      <c r="F7" s="11">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -997,7 +954,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1006,32 +963,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
         <v>42</v>
-      </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="B3" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>